<commit_message>
Ok test search product
</commit_message>
<xml_diff>
--- a/data/data1.xlsx
+++ b/data/data1.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnTotNghiep_NguyenQuyen_10122312\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD5595B-7688-429F-A99C-923B2D50EEC3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552B321E-3B81-4206-888C-ED25478CAC4D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8010" activeTab="1" xr2:uid="{A15DE430-7E6B-4467-9607-107A07875CE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Search" sheetId="2" r:id="rId2"/>
+    <sheet name="Search" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
   <si>
     <t>TC</t>
   </si>
@@ -94,30 +94,6 @@
     <t>Login09</t>
   </si>
   <si>
-    <t>product</t>
-  </si>
-  <si>
-    <t>Search01</t>
-  </si>
-  <si>
-    <t>Search02</t>
-  </si>
-  <si>
-    <t>Search03</t>
-  </si>
-  <si>
-    <t>Search04</t>
-  </si>
-  <si>
-    <t>Search05</t>
-  </si>
-  <si>
-    <t>Search06</t>
-  </si>
-  <si>
-    <t>Vui lòng điền vào trường này</t>
-  </si>
-  <si>
     <t>5cm</t>
   </si>
   <si>
@@ -137,6 +113,15 @@
   </si>
   <si>
     <t>Giày sandal công sở ELLA 7cm thanh lịch cuốn hút ELA662</t>
+  </si>
+  <si>
+    <t>${product}</t>
+  </si>
+  <si>
+    <t>${expected}</t>
+  </si>
+  <si>
+    <t>Please fill out this field.</t>
   </si>
 </sst>
 </file>
@@ -637,85 +622,65 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B883B53-4143-4FF1-8D4F-E56E6C8DAA85}">
-  <dimension ref="A1:C7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667F2FF2-D70E-4CEB-89DF-FD887F6CFB59}">
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="3" width="22.26953125" customWidth="1"/>
+    <col min="1" max="1" width="20.26953125" customWidth="1"/>
+    <col min="2" max="2" width="24.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="B1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>22</v>
       </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>23</v>
       </c>
-      <c r="C2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>